<commit_message>
Corrección definitiva de alineación SIS Gastos v1.7.6
</commit_message>
<xml_diff>
--- a/assets/plantilla_SCOF01.xlsx
+++ b/assets/plantilla_SCOF01.xlsx
@@ -2780,8 +2780,8 @@
     <mergeCell ref="I62:J62"/>
     <mergeCell ref="I59:J59"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="1.135" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="5" scale="37" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
+  <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
   <extLst>

</xml_diff>